<commit_message>
Release portfolio-ready Book Content Monitor
</commit_message>
<xml_diff>
--- a/examples/output/part1_processed.xlsx
+++ b/examples/output/part1_processed.xlsx
@@ -462,7 +462,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Правообладатель</t>
+          <t>Праообладатель</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -559,12 +559,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder</t>
+          <t>Avery Demo</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>DemoBook Amber 101</t>
+          <t>DemoBook Aurora 101</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101</t>
+          <t>https://library.example/aurora-101</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -597,17 +597,17 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>demobook amber 101</t>
+          <t>demobook aurora 101</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101</t>
+          <t>https://library.example/aurora-101</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -617,17 +617,17 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>record_9a91b99c1d248def</t>
+          <t>record_e50aae306c670af9</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>url_7c9e1bac0b47e7ac</t>
+          <t>url_abded59889089114</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda</t>
+          <t>book_4e377ef9865aaadb</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
@@ -659,12 +659,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder</t>
+          <t>Avery Demo</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>DemoBook Amber 101</t>
+          <t>DemoBook Aurora 101</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101</t>
+          <t>https://library.example/aurora-101</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -697,17 +697,17 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>demobook amber 101</t>
+          <t>demobook aurora 101</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101</t>
+          <t>https://library.example/aurora-101</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -717,17 +717,17 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>record_9a91b99c1d248def</t>
+          <t>record_e50aae306c670af9</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>url_7c9e1bac0b47e7ac</t>
+          <t>url_abded59889089114</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda</t>
+          <t>book_4e377ef9865aaadb</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
@@ -759,12 +759,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder</t>
+          <t>Avery Demo</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>DemoBook Amber 101</t>
+          <t>DemoBook Aurora 101</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://s4.library.example/amber-101</t>
+          <t>https://s4.library.example/aurora-101</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>demobook amber 101</t>
+          <t>demobook aurora 101</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>https://s4.library.example/amber-101</t>
+          <t>https://s4.library.example/aurora-101</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -817,17 +817,17 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>record_b2b15d1274cb2e76</t>
+          <t>record_78a339a07f162aa7</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>url_02c4ada8a33c4916</t>
+          <t>url_3d96402c20f4bcf4</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda</t>
+          <t>book_4e377ef9865aaadb</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Owen Sample</t>
+          <t>Robin Sample</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>DemoBook Amber 101</t>
+          <t>DemoBook Aurora 101</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101</t>
+          <t>https://library.example/aurora-101</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -893,17 +893,17 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>owen sample</t>
+          <t>robin sample</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>demobook amber 101</t>
+          <t>demobook aurora 101</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101</t>
+          <t>https://library.example/aurora-101</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -913,17 +913,17 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>record_3bb7e8c5167a5248</t>
+          <t>record_ccd64917f5c65f19</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>url_7c9e1bac0b47e7ac</t>
+          <t>url_abded59889089114</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>book_92e8609287835043</t>
+          <t>book_e60bb9056ea7db02</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -952,12 +952,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder</t>
+          <t>Avery Demo</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>DemoBook Amber 101</t>
+          <t>DemoBook Aurora 101</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101-audio</t>
+          <t>https://library.example/aurora-101-audio</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -990,17 +990,17 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>demobook amber 101</t>
+          <t>demobook aurora 101</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101-audio</t>
+          <t>https://library.example/aurora-101-audio</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -1010,17 +1010,17 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>record_2a9ffd1dc4147192</t>
+          <t>record_556ddd03f596d1aa</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>url_4711f6189586f4f2</t>
+          <t>url_472faf3c0a87b7b8</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>book_2e7d1df11b480472</t>
+          <t>book_5426806284eb9cc9</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder</t>
+          <t>Avery Demo</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/authors/mira</t>
+          <t>https://library.example/authors/avery</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/authors/mira</t>
+          <t>https://library.example/authors/avery</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1649,17 +1649,17 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>record_a56e4d080c663d2d</t>
+          <t>record_f1821837fdba956e</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>url_e51266190d9b84c6</t>
+          <t>url_69a44ed23c109e21</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>book_8d8a37fa567d2e57</t>
+          <t>book_f07d5c2030a60ddf</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Owen Sample</t>
+          <t>Robin Sample</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>owen sample</t>
+          <t>robin sample</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>record_1e1b80aac927bf72</t>
+          <t>record_3f70afb68b334b6e</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>book_4c77c68a9661926a</t>
+          <t>book_7bfa8256e8598741</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
@@ -1951,12 +1951,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder</t>
+          <t>Avery Demo</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Demo Amber Room</t>
+          <t>Demo Aurora Room</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1989,12 +1989,12 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>demo amber room</t>
+          <t>demo aurora room</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>record_72740d395997b0fd</t>
+          <t>record_316badd0cea45473</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>book_67e268643fb6e40e</t>
+          <t>book_6e0a0b0dbae03161</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder;</t>
+          <t>Avery Demo;</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>record_0366d1bf1ee75fba</t>
+          <t>record_2e4829f002f0dd4e</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>book_9707fc4afab8d394</t>
+          <t>book_50f21b3560eafd9e</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Owen Sample</t>
+          <t>Robin Sample</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>owen sample</t>
+          <t>robin sample</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>record_9b1c536097e7c77a</t>
+          <t>record_b7d4a9ae67f29888</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>book_dc6f530713a65e12</t>
+          <t>book_2abb8e2a34cc1a89</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>record_9a91b99c1d248def</t>
+          <t>record_e50aae306c670af9</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2301,12 +2301,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda</t>
+          <t>book_4e377ef9865aaadb</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101</t>
+          <t>https://library.example/aurora-101</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>url_7c9e1bac0b47e7ac</t>
+          <t>url_abded59889089114</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2341,13 +2341,13 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda
-book_92e8609287835043</t>
+          <t>book_4e377ef9865aaadb
+book_e60bb9056ea7db02</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101</t>
+          <t>https://library.example/aurora-101</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda</t>
+          <t>book_4e377ef9865aaadb</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2422,13 +2422,13 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda</t>
+          <t>book_4e377ef9865aaadb</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101
-https://s4.library.example/amber-101</t>
+          <t>https://library.example/aurora-101
+https://s4.library.example/aurora-101</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -2537,17 +2537,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda</t>
+          <t>book_4e377ef9865aaadb</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>demobook amber 101</t>
+          <t>demobook aurora 101</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2570,18 +2570,18 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101
-https://s4.library.example/amber-101</t>
+          <t>https://library.example/aurora-101
+https://s4.library.example/aurora-101</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder</t>
+          <t>Avery Demo</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>DemoBook Amber 101</t>
+          <t>DemoBook Aurora 101</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2609,17 +2609,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>book_92e8609287835043</t>
+          <t>book_e60bb9056ea7db02</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>owen sample</t>
+          <t>robin sample</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>demobook amber 101</t>
+          <t>demobook aurora 101</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2640,17 +2640,17 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101</t>
+          <t>https://library.example/aurora-101</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Owen Sample</t>
+          <t>Robin Sample</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>DemoBook Amber 101</t>
+          <t>DemoBook Aurora 101</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2675,17 +2675,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>book_2e7d1df11b480472</t>
+          <t>book_5426806284eb9cc9</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>demobook amber 101</t>
+          <t>demobook aurora 101</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2706,17 +2706,17 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/amber-101-audio</t>
+          <t>https://library.example/aurora-101-audio</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder</t>
+          <t>Avery Demo</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>DemoBook Amber 101</t>
+          <t>DemoBook Aurora 101</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -3119,12 +3119,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>book_8d8a37fa567d2e57</t>
+          <t>book_f07d5c2030a60ddf</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -3150,12 +3150,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>https://library.example/authors/mira</t>
+          <t>https://library.example/authors/avery</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder</t>
+          <t>Avery Demo</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -3182,12 +3182,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>book_4c77c68a9661926a</t>
+          <t>book_7bfa8256e8598741</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>owen sample</t>
+          <t>robin sample</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Owen Sample</t>
+          <t>Robin Sample</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -3371,17 +3371,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>book_67e268643fb6e40e</t>
+          <t>book_6e0a0b0dbae03161</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>demo amber room</t>
+          <t>demo aurora room</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -3407,12 +3407,12 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder</t>
+          <t>Avery Demo</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Demo Amber Room</t>
+          <t>Demo Aurora Room</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -3434,12 +3434,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>book_9707fc4afab8d394</t>
+          <t>book_50f21b3560eafd9e</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>mira placeholder</t>
+          <t>avery demo</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Mira Placeholder;</t>
+          <t>Avery Demo;</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -3493,12 +3493,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>book_dc6f530713a65e12</t>
+          <t>book_2abb8e2a34cc1a89</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>owen sample</t>
+          <t>robin sample</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Owen Sample</t>
+          <t>Robin Sample</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Слабое сходство названия с текстом URL (покрытие слов 38%). Возможны другое произведение, иной подзаголовок или другая транслитерация.</t>
+          <t>Слабое сходство названия с текстом URL (покрытие слов 43%). Возможны другое произведение, иной подзаголовок или другая транслитерация.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda</t>
+          <t>book_4e377ef9865aaadb</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Слабое сходство названия с текстом URL (покрытие слов 38%). Возможны другое произведение, иной подзаголовок или другая транслитерация.</t>
+          <t>Слабое сходство названия с текстом URL (покрытие слов 43%). Возможны другое произведение, иной подзаголовок или другая транслитерация.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda</t>
+          <t>book_4e377ef9865aaadb</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Слабое сходство названия с текстом URL (покрытие слов 38%). Возможны другое произведение, иной подзаголовок или другая транслитерация.</t>
+          <t>Слабое сходство названия с текстом URL (покрытие слов 43%). Возможны другое произведение, иной подзаголовок или другая транслитерация.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda</t>
+          <t>book_4e377ef9865aaadb</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Слабое сходство названия с текстом URL (покрытие слов 38%). Возможны другое произведение, иной подзаголовок или другая транслитерация.</t>
+          <t>Слабое сходство названия с текстом URL (покрытие слов 43%). Возможны другое произведение, иной подзаголовок или другая транслитерация.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -3753,7 +3753,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>book_92e8609287835043</t>
+          <t>book_e60bb9056ea7db02</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Слабое сходство названия с текстом URL (покрытие слов 38%). Возможны другое произведение, иной подзаголовок или другая транслитерация.</t>
+          <t>Слабое сходство названия с текстом URL (покрытие слов 43%). Возможны другое произведение, иной подзаголовок или другая транслитерация.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>book_2e7d1df11b480472</t>
+          <t>book_5426806284eb9cc9</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>book_8d8a37fa567d2e57</t>
+          <t>book_f07d5c2030a60ddf</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>book_4c77c68a9661926a</t>
+          <t>book_7bfa8256e8598741</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -4123,7 +4123,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>book_67e268643fb6e40e</t>
+          <t>book_6e0a0b0dbae03161</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -4160,7 +4160,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>book_dc6f530713a65e12</t>
+          <t>book_2abb8e2a34cc1a89</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -4275,9 +4275,9 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>book_2e7d1df11b480472
-book_74e3f59c074a5cda
-book_92e8609287835043</t>
+          <t>book_4e377ef9865aaadb
+book_5426806284eb9cc9
+book_e60bb9056ea7db02</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4356,8 +4356,8 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>book_2e7d1df11b480472
-book_74e3f59c074a5cda</t>
+          <t>book_4e377ef9865aaadb
+book_5426806284eb9cc9</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4476,8 +4476,8 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda
-book_92e8609287835043</t>
+          <t>book_4e377ef9865aaadb
+book_e60bb9056ea7db02</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -4556,8 +4556,8 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>book_74e3f59c074a5cda
-book_92e8609287835043</t>
+          <t>book_4e377ef9865aaadb
+book_e60bb9056ea7db02</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">

</xml_diff>